<commit_message>
Enhance lab and quiz consolidation script with logging and improved data handling
- Updated the script to use logging instead of print statements for better tracking of the process.
- Modified the file path for the Excel file to reflect the correct naming convention.
- Added functionality to read all sheets from the Excel file and differentiate between Labs and Quizzes.
- Introduced a 'marks_type' column to indicate whether the score is from a Lab or a Quiz.
- Improved error handling and warnings for missing files and sheets without 'Week' columns.
- Ensured the output CSV file is saved with the correct structure and metadata.
</commit_message>
<xml_diff>
--- a/Module 8 Data/Cloud Training/Labs & Quizes/labs_and_quizzes.xlsx
+++ b/Module 8 Data/Cloud Training/Labs & Quizes/labs_and_quizzes.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amalitech-my.sharepoint.com/personal/ernest_kwisanga_amalitech_com/Documents/Desktop/Moodle Labs/Specilization/DEM08/Module 8 Data/Cloud Training/Labs &amp; Quizes/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_4FE271004603599242870A3343FDE641CA53328B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54731798-E5BE-4209-B83A-DB8F5DA6F160}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Labs" sheetId="1" r:id="rId1"/>
     <sheet name="Quizzes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -173,8 +179,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,13 +243,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -281,7 +295,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -315,6 +329,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -349,9 +364,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -524,11 +540,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -563,7 +582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -598,7 +617,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -633,7 +652,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -668,7 +687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -703,7 +722,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -738,7 +757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -773,7 +792,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -808,7 +827,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -843,7 +862,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -878,7 +897,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -913,7 +932,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -948,7 +967,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -983,7 +1002,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1018,7 +1037,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1053,7 +1072,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1088,7 +1107,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1123,7 +1142,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1158,7 +1177,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1193,7 +1212,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1228,7 +1247,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1263,7 +1282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1298,7 +1317,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1333,7 +1352,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -1368,7 +1387,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -1403,7 +1422,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -1438,7 +1457,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -1473,7 +1492,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1508,7 +1527,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -1543,7 +1562,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -1578,7 +1597,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -1613,7 +1632,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1648,7 +1667,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1683,7 +1702,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -1718,7 +1737,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -1753,7 +1772,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -1788,7 +1807,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>46</v>
       </c>
@@ -1823,7 +1842,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -1858,7 +1877,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -1893,7 +1912,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -1928,7 +1947,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>
@@ -1969,11 +1988,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2008,7 +2027,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2043,7 +2062,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2078,7 +2097,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -2113,7 +2132,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -2148,7 +2167,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -2183,7 +2202,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2218,7 +2237,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -2253,7 +2272,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -2288,7 +2307,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2323,7 +2342,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -2358,7 +2377,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -2393,7 +2412,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -2428,7 +2447,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -2463,7 +2482,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -2498,7 +2517,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -2533,7 +2552,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -2568,7 +2587,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -2603,7 +2622,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -2638,7 +2657,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -2673,7 +2692,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -2708,7 +2727,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -2743,7 +2762,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -2778,7 +2797,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -2813,7 +2832,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -2848,7 +2867,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -2883,7 +2902,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -2918,7 +2937,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -2953,7 +2972,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -2988,7 +3007,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -3023,7 +3042,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -3058,7 +3077,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -3093,7 +3112,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -3128,7 +3147,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -3163,7 +3182,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -3198,7 +3217,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -3233,7 +3252,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>46</v>
       </c>
@@ -3268,7 +3287,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -3303,7 +3322,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -3338,7 +3357,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -3373,7 +3392,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>
@@ -3411,4 +3430,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{2f70ad68-4eca-4ffe-ad9d-60bfae449e23}" enabled="1" method="Standard" siteId="{b20a8f4d-0d6a-4f2e-83a2-181c968f8882}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>